<commit_message>
Support negative rubric weights
</commit_message>
<xml_diff>
--- a/rubric_template.xlsx
+++ b/rubric_template.xlsx
@@ -609,12 +609,12 @@
     <dataValidation sqref="B2:B501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Pick Content, Execution, or Presentation &amp; Formatting" prompt="Choose a category" type="list">
       <formula1>"Content,Execution,Presentation &amp; Formatting"</formula1>
     </dataValidation>
-    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Weight must be a whole number from 1 to 10" prompt="Enter a weight from 1 to 10" type="whole" operator="between">
-      <formula1>1</formula1>
-      <formula2>10</formula2>
-    </dataValidation>
     <dataValidation sqref="D2:D501 E2:E501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" prompt="Pass or Fail (leave blank for unset)" type="list">
       <formula1>"Pass,Fail"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Invalid weight" error="Enter a whole-number weight from -10 to 10." promptTitle="Rubric weight" prompt="Use a whole-number weight from -10 to 10. Negative weights are penalties when passed." type="whole" operator="between">
+      <formula1>-10</formula1>
+      <formula2>10</formula2>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -660,11 +660,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Total weight</t>
+          <t>Max positive weight</t>
         </is>
       </c>
       <c r="B3">
-        <f>SUM(Rubric!C2:C501)</f>
+        <f>SUMIF(Rubric!C2:C501,"&gt;0",Rubric!C2:C501)</f>
         <v/>
       </c>
     </row>

</xml_diff>